<commit_message>
Migrate to Google Sheets, harden call flow, add cloud scheduling
- Replace the local Excel backend with the live Google Sheets API so the
  schedule matches the task's stated input and stays readable/writable
  from anywhere.
- Add --once mode plus a GitHub Actions cron workflow, so reminders no
  longer depend on a laptop staying awake.
- Warm up the Render webhook before dialling. On the free tier the server
  sleeps after ~15 min; the cold start outlasted Twilio's ~15s webhook
  timeout, so the driver heard an error message instead of the reminder.
- Build TwiML with Twilio's VoiceResponse so a name or location
  containing & or < can no longer break the XML, and turn off Flask
  debug by default.
- Stop reporting a failed status fetch as "completed", which could mark
  an unanswered call as Sent.
- Add .gitignore (keeps .env and service_account.json out of the repo).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sample_Driver_Pickup_Schedule V2.xlsx
+++ b/Sample_Driver_Pickup_Schedule V2.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\singh\Desktop\mr cabie assignment\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C1CD6A2-F19A-4C7C-86BF-BEF02AC505EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sample_Driver_Pickup_Schedule V" sheetId="1" r:id="rId5"/>
+    <sheet name="Sample_Driver_Pickup_Schedule V" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
   <si>
     <t>Driver Name</t>
   </si>
@@ -74,23 +83,27 @@
   </si>
   <si>
     <t>New Delhi</t>
+  </si>
+  <si>
+    <t>Sent</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -101,43 +114,45 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -327,17 +342,23 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="18.21875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -354,7 +375,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -365,13 +386,13 @@
         <v>7</v>
       </c>
       <c r="D2" s="2">
-        <v>46252.902083333334</v>
+        <v>46252.902083333327</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -382,13 +403,13 @@
         <v>11</v>
       </c>
       <c r="D3" s="2">
-        <v>46252.916666666664</v>
+        <v>46252.916666666657</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -405,7 +426,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -422,7 +443,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -433,13 +454,16 @@
         <v>20</v>
       </c>
       <c r="D6" s="2">
-        <v>46252.90625</v>
+        <v>46253.038164513891</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>8</v>
-      </c>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D7" s="3"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Never dial a ride whose outcome cannot be recorded
A live test exposed a real failure: the call went out, then the status
write-back hit "[Errno 13] Permission denied" because the workbook was
open in Excel. The row stayed "Pending" and was still inside the reminder
window, so the next cycle would have called the driver again - and again
every cycle until the window closed.

- sheet_handler.can_write() reports whether the status can be persisted.
  For Excel that means no "~$" sidecar lock and the file opening for
  write; the agent skips the cycle with a clear message instead of
  dialling.
- Rows dialled during a run are remembered, so even a write that fails
  after the call cannot cause a repeat dial.
- A failed write is reported instead of crashing the whole cycle.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sample_Driver_Pickup_Schedule V2.xlsx
+++ b/Sample_Driver_Pickup_Schedule V2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\singh\Desktop\mr cabie assignment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C1CD6A2-F19A-4C7C-86BF-BEF02AC505EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{868904F7-098B-426C-A397-BE936F4FE5F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>Driver Name</t>
   </si>
@@ -83,9 +83,6 @@
   </si>
   <si>
     <t>New Delhi</t>
-  </si>
-  <si>
-    <t>Sent</t>
   </si>
 </sst>
 </file>
@@ -454,10 +451,10 @@
         <v>20</v>
       </c>
       <c r="D6" s="2">
-        <v>46253.038164513891</v>
+        <v>46253.584722222222</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>